<commit_message>
add vv labels; start cleaning
</commit_message>
<xml_diff>
--- a/ext/var_labels_who_survey.xlsx
+++ b/ext/var_labels_who_survey.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chegu\Documents\R\mend-wc\ext\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roberto Mediavilla\Documents\r-projects\mend-gps\ext\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA9DACB-5B91-487C-ACD4-89EC23BECEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E1FD6A6-2FB7-4E15-B8BB-151F8D217A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="384">
   <si>
     <t>Question_uuid</t>
   </si>
@@ -1176,6 +1176,18 @@
   </si>
   <si>
     <t>Probable alcohol dependence</t>
+  </si>
+  <si>
+    <t>phqads_z</t>
+  </si>
+  <si>
+    <t>PHQ-ADS score (Z)</t>
+  </si>
+  <si>
+    <t>phqads_sc</t>
+  </si>
+  <si>
+    <t>PHQ-ADS score (observed)</t>
   </si>
 </sst>
 </file>
@@ -1247,7 +1259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1281,6 +1293,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1360,8 +1375,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BC2CEF76-BACA-45DC-A105-02C6E84761C4}" name="Tabla1" displayName="Tabla1" ref="A1:C158" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:C158" xr:uid="{BC2CEF76-BACA-45DC-A105-02C6E84761C4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BC2CEF76-BACA-45DC-A105-02C6E84761C4}" name="Tabla1" displayName="Tabla1" ref="A1:C160" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:C160" xr:uid="{BC2CEF76-BACA-45DC-A105-02C6E84761C4}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{6AEDBD45-3B2C-4BF6-91BA-E9C50FD7AB94}" name="Question_uuid" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{E6E57A5C-3751-4E7C-8476-A4B8715801C7}" name="Question" dataDxfId="1"/>
@@ -1688,15 +1703,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E158"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E160"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="42" style="5" customWidth="1"/>
-    <col min="3" max="3" width="45.1796875" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.140625" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1707,7 +1722,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1718,7 +1733,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -1729,7 +1744,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>216</v>
       </c>
@@ -1740,7 +1755,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="5" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>219</v>
       </c>
@@ -1751,7 +1766,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="6" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
@@ -1762,7 +1777,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
@@ -1773,7 +1788,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
@@ -1784,7 +1799,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
@@ -1795,7 +1810,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>17</v>
       </c>
@@ -1806,7 +1821,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>20</v>
       </c>
@@ -1817,7 +1832,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>297</v>
       </c>
@@ -1826,7 +1841,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>23</v>
       </c>
@@ -1837,7 +1852,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>26</v>
       </c>
@@ -1848,7 +1863,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>29</v>
       </c>
@@ -1859,7 +1874,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>32</v>
       </c>
@@ -1870,7 +1885,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>35</v>
       </c>
@@ -1881,7 +1896,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>38</v>
       </c>
@@ -1892,7 +1907,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>41</v>
       </c>
@@ -1903,7 +1918,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>43</v>
       </c>
@@ -1914,7 +1929,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -1925,7 +1940,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>49</v>
       </c>
@@ -1936,7 +1951,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>52</v>
       </c>
@@ -1947,7 +1962,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>55</v>
       </c>
@@ -1958,7 +1973,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>58</v>
       </c>
@@ -1969,7 +1984,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>60</v>
       </c>
@@ -1980,7 +1995,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>62</v>
       </c>
@@ -1991,7 +2006,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="87" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" ht="105" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>64</v>
       </c>
@@ -2002,7 +2017,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>66</v>
       </c>
@@ -2013,7 +2028,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>69</v>
       </c>
@@ -2024,7 +2039,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>72</v>
       </c>
@@ -2035,7 +2050,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>75</v>
       </c>
@@ -2046,7 +2061,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>77</v>
       </c>
@@ -2057,7 +2072,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>79</v>
       </c>
@@ -2068,7 +2083,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>82</v>
       </c>
@@ -2079,7 +2094,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>84</v>
       </c>
@@ -2090,7 +2105,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>87</v>
       </c>
@@ -2101,7 +2116,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>90</v>
       </c>
@@ -2112,7 +2127,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>92</v>
       </c>
@@ -2123,7 +2138,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>94</v>
       </c>
@@ -2134,7 +2149,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>96</v>
       </c>
@@ -2145,7 +2160,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>98</v>
       </c>
@@ -2156,7 +2171,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>101</v>
       </c>
@@ -2167,7 +2182,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>104</v>
       </c>
@@ -2178,7 +2193,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>107</v>
       </c>
@@ -2189,7 +2204,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>109</v>
       </c>
@@ -2200,7 +2215,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>112</v>
       </c>
@@ -2211,7 +2226,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>114</v>
       </c>
@@ -2222,7 +2237,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>116</v>
       </c>
@@ -2233,7 +2248,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>118</v>
       </c>
@@ -2244,7 +2259,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>120</v>
       </c>
@@ -2255,7 +2270,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>122</v>
       </c>
@@ -2266,7 +2281,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>124</v>
       </c>
@@ -2277,7 +2292,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>126</v>
       </c>
@@ -2288,7 +2303,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>128</v>
       </c>
@@ -2299,7 +2314,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>130</v>
       </c>
@@ -2310,7 +2325,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>133</v>
       </c>
@@ -2321,7 +2336,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>136</v>
       </c>
@@ -2332,7 +2347,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>139</v>
       </c>
@@ -2343,7 +2358,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>142</v>
       </c>
@@ -2355,7 +2370,7 @@
       </c>
       <c r="E60" s="8"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>145</v>
       </c>
@@ -2366,7 +2381,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>148</v>
       </c>
@@ -2377,7 +2392,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>150</v>
       </c>
@@ -2388,7 +2403,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>153</v>
       </c>
@@ -2399,7 +2414,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>156</v>
       </c>
@@ -2410,7 +2425,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>159</v>
       </c>
@@ -2421,7 +2436,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>161</v>
       </c>
@@ -2432,7 +2447,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>163</v>
       </c>
@@ -2443,7 +2458,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>165</v>
       </c>
@@ -2454,7 +2469,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>167</v>
       </c>
@@ -2465,7 +2480,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>169</v>
       </c>
@@ -2476,7 +2491,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>172</v>
       </c>
@@ -2487,7 +2502,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>175</v>
       </c>
@@ -2498,7 +2513,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>178</v>
       </c>
@@ -2509,7 +2524,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>181</v>
       </c>
@@ -2520,7 +2535,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>184</v>
       </c>
@@ -2531,7 +2546,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>186</v>
       </c>
@@ -2542,7 +2557,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>188</v>
       </c>
@@ -2553,7 +2568,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>190</v>
       </c>
@@ -2564,7 +2579,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>193</v>
       </c>
@@ -2575,7 +2590,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>196</v>
       </c>
@@ -2586,7 +2601,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>199</v>
       </c>
@@ -2597,7 +2612,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>202</v>
       </c>
@@ -2608,7 +2623,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
         <v>205</v>
       </c>
@@ -2619,7 +2634,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>207</v>
       </c>
@@ -2630,7 +2645,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
         <v>210</v>
       </c>
@@ -2641,7 +2656,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="116" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" ht="135" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>213</v>
       </c>
@@ -2652,7 +2667,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>222</v>
       </c>
@@ -2661,7 +2676,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
         <v>223</v>
       </c>
@@ -2670,7 +2685,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
         <v>224</v>
       </c>
@@ -2679,7 +2694,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>225</v>
       </c>
@@ -2688,7 +2703,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
         <v>226</v>
       </c>
@@ -2697,7 +2712,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
         <v>227</v>
       </c>
@@ -2706,7 +2721,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
         <v>228</v>
       </c>
@@ -2715,7 +2730,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>229</v>
       </c>
@@ -2724,7 +2739,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
         <v>230</v>
       </c>
@@ -2733,7 +2748,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
         <v>231</v>
       </c>
@@ -2742,7 +2757,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
         <v>232</v>
       </c>
@@ -2751,7 +2766,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
         <v>233</v>
       </c>
@@ -2760,7 +2775,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
         <v>234</v>
       </c>
@@ -2769,7 +2784,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>235</v>
       </c>
@@ -2778,7 +2793,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="9" t="s">
         <v>303</v>
       </c>
@@ -2787,7 +2802,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
         <v>236</v>
       </c>
@@ -2796,7 +2811,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="6" t="s">
         <v>237</v>
       </c>
@@ -2805,7 +2820,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
         <v>238</v>
       </c>
@@ -2814,7 +2829,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
         <v>239</v>
       </c>
@@ -2823,7 +2838,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="9" t="s">
         <v>248</v>
       </c>
@@ -2832,7 +2847,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="6" t="s">
         <v>240</v>
       </c>
@@ -2841,7 +2856,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="6" t="s">
         <v>241</v>
       </c>
@@ -2850,7 +2865,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="9" t="s">
         <v>253</v>
       </c>
@@ -2859,7 +2874,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A111" s="6" t="s">
         <v>242</v>
       </c>
@@ -2868,7 +2883,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A112" s="6" t="s">
         <v>243</v>
       </c>
@@ -2877,7 +2892,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="9" t="s">
         <v>252</v>
       </c>
@@ -2886,7 +2901,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="6" t="s">
         <v>244</v>
       </c>
@@ -2895,7 +2910,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="6" t="s">
         <v>245</v>
       </c>
@@ -2904,7 +2919,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
         <v>246</v>
       </c>
@@ -2913,7 +2928,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
         <v>247</v>
       </c>
@@ -2922,7 +2937,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="9" t="s">
         <v>249</v>
       </c>
@@ -2931,7 +2946,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="9" t="s">
         <v>251</v>
       </c>
@@ -2940,7 +2955,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="6" t="s">
         <v>292</v>
       </c>
@@ -2949,7 +2964,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="6" t="s">
         <v>304</v>
       </c>
@@ -2958,7 +2973,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A122" s="6" t="s">
         <v>305</v>
       </c>
@@ -2967,7 +2982,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A123" s="9" t="s">
         <v>340</v>
       </c>
@@ -2976,7 +2991,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A124" s="6" t="s">
         <v>308</v>
       </c>
@@ -2985,7 +3000,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="9" t="s">
         <v>341</v>
       </c>
@@ -2994,7 +3009,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="9" t="s">
         <v>342</v>
       </c>
@@ -3003,7 +3018,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="9" t="s">
         <v>343</v>
       </c>
@@ -3012,7 +3027,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="9" t="s">
         <v>344</v>
       </c>
@@ -3021,7 +3036,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="9" t="s">
         <v>311</v>
       </c>
@@ -3030,7 +3045,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="9" t="s">
         <v>313</v>
       </c>
@@ -3039,7 +3054,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="9" t="s">
         <v>318</v>
       </c>
@@ -3048,7 +3063,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="6" t="s">
         <v>314</v>
       </c>
@@ -3057,7 +3072,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="6" t="s">
         <v>315</v>
       </c>
@@ -3066,7 +3081,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="6" t="s">
         <v>316</v>
       </c>
@@ -3075,7 +3090,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="9" t="s">
         <v>319</v>
       </c>
@@ -3084,7 +3099,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" s="9" t="s">
         <v>320</v>
       </c>
@@ -3093,7 +3108,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" s="9" t="s">
         <v>378</v>
       </c>
@@ -3102,7 +3117,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" s="9" t="s">
         <v>321</v>
       </c>
@@ -3111,7 +3126,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" s="9" t="s">
         <v>322</v>
       </c>
@@ -3120,7 +3135,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" s="9" t="s">
         <v>323</v>
       </c>
@@ -3129,7 +3144,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" s="9" t="s">
         <v>324</v>
       </c>
@@ -3138,7 +3153,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" s="9" t="s">
         <v>325</v>
       </c>
@@ -3147,7 +3162,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" s="9" t="s">
         <v>326</v>
       </c>
@@ -3156,7 +3171,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" s="9" t="s">
         <v>327</v>
       </c>
@@ -3165,7 +3180,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="9" t="s">
         <v>328</v>
       </c>
@@ -3174,7 +3189,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" s="9" t="s">
         <v>329</v>
       </c>
@@ -3183,7 +3198,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" s="9" t="s">
         <v>330</v>
       </c>
@@ -3192,7 +3207,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" s="9" t="s">
         <v>331</v>
       </c>
@@ -3201,7 +3216,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" s="9" t="s">
         <v>351</v>
       </c>
@@ -3210,7 +3225,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" s="9" t="s">
         <v>352</v>
       </c>
@@ -3219,7 +3234,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" s="6" t="s">
         <v>349</v>
       </c>
@@ -3228,7 +3243,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" s="6" t="s">
         <v>350</v>
       </c>
@@ -3237,7 +3252,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A153" s="9" t="s">
         <v>354</v>
       </c>
@@ -3246,7 +3261,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" s="9" t="s">
         <v>355</v>
       </c>
@@ -3255,7 +3270,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" s="6" t="s">
         <v>356</v>
       </c>
@@ -3264,7 +3279,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" s="9" t="s">
         <v>361</v>
       </c>
@@ -3273,7 +3288,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" s="9" t="s">
         <v>251</v>
       </c>
@@ -3282,7 +3297,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" s="6" t="s">
         <v>363</v>
       </c>
@@ -3291,10 +3306,29 @@
         <v>367</v>
       </c>
     </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="B159" s="2"/>
+      <c r="C159" s="10" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A160" s="9" t="s">
+        <v>382</v>
+      </c>
+      <c r="B160" s="2"/>
+      <c r="C160" s="12" t="s">
+        <v>383</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>